<commit_message>
Final verified: Excel files updated, Python scripts added, PowerPoint aligned with model
</commit_message>
<xml_diff>
--- a/data/competitor_benchmarking.xlsx
+++ b/data/competitor_benchmarking.xlsx
@@ -1,113 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dialog axiata financial Analyst\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C6F511-92DF-457E-81BD-3DBBBE0A38C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Market Cap (USD Mn)</t>
-  </si>
-  <si>
-    <t>Revenue (USD Mn)</t>
-  </si>
-  <si>
-    <t>EBITDA (USD Mn)</t>
-  </si>
-  <si>
-    <t>Net Margin %</t>
-  </si>
-  <si>
-    <t>EBITDA Margin %</t>
-  </si>
-  <si>
-    <t>Debt/Equity</t>
-  </si>
-  <si>
-    <t>ROE %</t>
-  </si>
-  <si>
-    <t>P/E Ratio</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Dialog Axiata (LK)</t>
-  </si>
-  <si>
-    <t>Dialog Axiata Annual Report 2024 (PDF verified)</t>
-  </si>
-  <si>
-    <t>Axiata Group (MY)</t>
-  </si>
-  <si>
-    <t>yfinance · 6888.KL · FX: 1 MYR = 0.223714 USD</t>
-  </si>
-  <si>
-    <t>Bharti Airtel (IN)</t>
-  </si>
-  <si>
-    <t>yfinance · BHARTIARTL.NS · FX: 1 INR = 0.011976 USD</t>
-  </si>
-  <si>
-    <t>Indosat (ID)</t>
-  </si>
-  <si>
-    <t>yfinance · ISAT.JK · FX: 1 IDR = 0.000063 USD</t>
-  </si>
-  <si>
-    <t>Telkom Indonesia</t>
-  </si>
-  <si>
-    <t>yfinance · TLKM.JK · FX: 1 IDR = 0.000063 USD</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -141,26 +66,85 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{BBEA2724-811A-48AD-98F1-FB20053AE08D}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0"/>
   </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -448,212 +432,275 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.33203125" bestFit="1" customWidth="1"/>
+    <col width="15.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="19.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="17.21875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="15.88671875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="15.5546875" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="11.21875" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="6.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="8.77734375" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="45.33203125" bestFit="1" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Market Cap (USD Mn)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue (USD Mn)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA (USD Mn)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Net Margin %</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA Margin %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Debt/Equity</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ROE %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>P/E Ratio</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dialog Axiata (LK)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>233</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>570.6</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>220.9</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>7.26</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>38.72</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>1.38</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="n">
         <v>15.89</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="n">
         <v>5.62</v>
       </c>
-      <c r="J2" t="s">
-        <v>11</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Dialog Axiata Annual Report 2024 (PDF verified)</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Axiata Group (MY)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>4645.5</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>2630.4</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>1115.8</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>3.1</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>42.42</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>70.03</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="n">
         <v>1.31</v>
       </c>
-      <c r="I3">
+      <c r="I3" t="n">
         <v>226</v>
       </c>
-      <c r="J3" t="s">
-        <v>13</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>yfinance · 6888.KL · FX: 1 MYR = 0.223714 USD</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bharti Airtel (IN)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>130561.8</v>
       </c>
-      <c r="C4">
-        <v>24367.200000000001</v>
-      </c>
-      <c r="D4">
+      <c r="C4" t="n">
+        <v>24367.2</v>
+      </c>
+      <c r="D4" t="n">
         <v>12678.6</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>14.94</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>52.03</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>117.09</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="n">
         <v>23.12</v>
       </c>
-      <c r="I4">
+      <c r="I4" t="n">
         <v>35.21</v>
       </c>
-      <c r="J4" t="s">
-        <v>15</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>yfinance · BHARTIARTL.NS · FX: 1 INR = 0.011976 USD</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Indosat (ID)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>4245.7</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>3577.1</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>1329.2</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>9.75</v>
       </c>
-      <c r="F5">
-        <v>37.159999999999997</v>
-      </c>
-      <c r="G5">
+      <c r="F5" t="n">
+        <v>37.16</v>
+      </c>
+      <c r="G5" t="n">
         <v>138.99</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="n">
         <v>15.28</v>
       </c>
-      <c r="I5">
+      <c r="I5" t="n">
         <v>12.18</v>
       </c>
-      <c r="J5" t="s">
-        <v>17</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>yfinance · ISAT.JK · FX: 1 IDR = 0.000063 USD</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Telkom Indonesia</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>19624.3</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>9326.9</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>3895.8</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>14.77</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>41.77</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>50.11</v>
       </c>
-      <c r="H6">
-        <v>18.309999999999999</v>
-      </c>
-      <c r="I6">
+      <c r="H6" t="n">
+        <v>18.31</v>
+      </c>
+      <c r="I6" t="n">
         <v>14.27</v>
       </c>
-      <c r="J6" t="s">
-        <v>19</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>yfinance · TLKM.JK · FX: 1 IDR = 0.000063 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>66276</v>
+      </c>
+      <c r="B7" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-18.8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>171.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>66276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>